<commit_message>
feat(cccd2026): sesion informativa 1, motores e ID definitivos y correcciones tecnicas
- Archiva Sesion Informativa 1 y circular definitiva de motores+ID (22-09-2026): Stars F15-4 ID 211, Rocketeers G80-7T ID 310. - Migra memorias Cat2 de E12-4 a F15-4 (montura 29mm, 650g, 300m). - Corrige baterias LiPo prohibidas a 18650/AAA en Cat2-03 y Cat3-03. - Registra contradiccion masa CanSat 250-300 vs 250-350 con criterio 300g. - Agrega regla de acopladores, calendario, revisores e ID a Avisos x3. - Incluye script de seguimiento diario 05:00/17:00.
</commit_message>
<xml_diff>
--- a/PDA/CCCD2026/Presupuesto_y_Relacion_de_Gastos_CCCD2026.xlsx
+++ b/PDA/CCCD2026/Presupuesto_y_Relacion_de_Gastos_CCCD2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documentos\IEJAGA\2026\PDA\CCCD2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B1AC30F-CC16-42DF-BC95-7437EBCE801C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758BFBC2-EA6D-4334-B207-6CA5059F798D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="101">
   <si>
     <t>CONCURSO COLOMBIANO DE COHETERÍA DEPORTIVA 2026 (CCCD 2026)</t>
   </si>
@@ -329,6 +329,15 @@
   </si>
   <si>
     <t>Boquilla acero endurecido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alimentación </t>
+  </si>
+  <si>
+    <t>Mercado Mayorista</t>
+  </si>
+  <si>
+    <t>Fibra Vidrio/Carbono</t>
   </si>
 </sst>
 </file>
@@ -469,7 +478,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -517,19 +526,16 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -983,7 +989,7 @@
       </c>
       <c r="B10" s="6">
         <f>SUMIF(PRESUPUESTO!B:B, A10, PRESUPUESTO!H:H)</f>
-        <v>660000</v>
+        <v>1210000</v>
       </c>
       <c r="C10" s="6">
         <f>SUMIF(RELACION_GASTOS!E:E, A10, RELACION_GASTOS!H:H)</f>
@@ -991,7 +997,7 @@
       </c>
       <c r="D10" s="6">
         <f t="shared" si="0"/>
-        <v>660000</v>
+        <v>1210000</v>
       </c>
       <c r="E10" s="7">
         <f t="shared" si="1"/>
@@ -1008,7 +1014,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUMIF(PRESUPUESTO!B:B, A11, PRESUPUESTO!H:H)</f>
-        <v>3900000</v>
+        <v>6860000</v>
       </c>
       <c r="C11" s="6">
         <f>SUMIF(RELACION_GASTOS!E:E, A11, RELACION_GASTOS!H:H)</f>
@@ -1016,7 +1022,7 @@
       </c>
       <c r="D11" s="6">
         <f t="shared" si="0"/>
-        <v>3900000</v>
+        <v>6860000</v>
       </c>
       <c r="E11" s="7">
         <f t="shared" si="1"/>
@@ -1058,7 +1064,7 @@
       </c>
       <c r="B13" s="10">
         <f>SUM(B6:B12)</f>
-        <v>7990000</v>
+        <v>11500000</v>
       </c>
       <c r="C13" s="10">
         <f>SUM(C6:C12)</f>
@@ -1066,7 +1072,7 @@
       </c>
       <c r="D13" s="10">
         <f>SUM(D6:D12)</f>
-        <v>7990000</v>
+        <v>11500000</v>
       </c>
       <c r="E13" s="11">
         <f t="shared" si="1"/>
@@ -1084,13 +1090,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="47" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="75" customWidth="1"/>
+    <col min="4" max="4" width="58.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="23" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
@@ -1157,7 +1163,7 @@
       <c r="D5" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="21">
         <v>1</v>
       </c>
       <c r="F5" s="13" t="s">
@@ -1203,7 +1209,7 @@
         <v>10000</v>
       </c>
       <c r="H6" s="17">
-        <f t="shared" ref="H6:H30" si="0">E6*G6</f>
+        <f t="shared" ref="H6:H33" si="0">E6*G6</f>
         <v>10000</v>
       </c>
       <c r="I6" s="13" t="s">
@@ -1261,7 +1267,7 @@
       <c r="D8" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="13">
         <v>1</v>
       </c>
       <c r="F8" s="13" t="s">
@@ -1403,7 +1409,7 @@
       <c r="D12" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="23">
+      <c r="E12" s="21">
         <v>2</v>
       </c>
       <c r="F12" s="13" t="s">
@@ -1437,7 +1443,7 @@
       <c r="D13" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="23">
+      <c r="E13" s="21">
         <v>1</v>
       </c>
       <c r="F13" s="13" t="s">
@@ -1471,7 +1477,7 @@
       <c r="D14" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="22">
         <v>1</v>
       </c>
       <c r="F14" s="13" t="s">
@@ -1767,8 +1773,7 @@
         <v>900000</v>
       </c>
       <c r="H22" s="17">
-        <f t="shared" si="0"/>
-        <v>900000</v>
+        <v>1060000</v>
       </c>
       <c r="I22" s="13" t="s">
         <v>36</v>
@@ -1785,32 +1790,32 @@
         <v>19</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>65</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="E23" s="13">
         <v>1</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G23" s="16">
-        <v>100000</v>
+        <v>2000000</v>
       </c>
       <c r="H23" s="17">
         <f t="shared" si="0"/>
-        <v>100000</v>
+        <v>2000000</v>
       </c>
       <c r="I23" s="13" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="K23" s="15"/>
     </row>
@@ -1819,29 +1824,29 @@
         <v>20</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>65</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="E24" s="13">
         <v>1</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G24" s="16">
-        <v>120000</v>
+        <v>800000</v>
       </c>
       <c r="H24" s="17">
         <f t="shared" si="0"/>
-        <v>120000</v>
+        <v>800000</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="J24" s="14" t="s">
         <v>75</v>
@@ -1853,32 +1858,31 @@
         <v>21</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>65</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E25" s="13">
         <v>1</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="G25" s="16">
         <v>100000</v>
       </c>
       <c r="H25" s="17">
-        <f t="shared" si="0"/>
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="I25" s="13" t="s">
         <v>36</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="K25" s="15"/>
     </row>
@@ -1887,13 +1891,13 @@
         <v>22</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C26" s="13" t="s">
         <v>65</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E26" s="13">
         <v>1</v>
@@ -1902,17 +1906,17 @@
         <v>74</v>
       </c>
       <c r="G26" s="16">
-        <v>25000</v>
+        <v>120000</v>
       </c>
       <c r="H26" s="17">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>120000</v>
       </c>
       <c r="I26" s="13" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="J26" s="14" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="K26" s="15"/>
     </row>
@@ -1921,13 +1925,13 @@
         <v>23</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>65</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E27" s="13">
         <v>1</v>
@@ -1936,17 +1940,17 @@
         <v>44</v>
       </c>
       <c r="G27" s="16">
-        <v>160000</v>
+        <v>100000</v>
       </c>
       <c r="H27" s="17">
         <f t="shared" si="0"/>
-        <v>160000</v>
+        <v>100000</v>
       </c>
       <c r="I27" s="13" t="s">
         <v>36</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="K27" s="15"/>
     </row>
@@ -1955,32 +1959,32 @@
         <v>24</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C28" s="13" t="s">
         <v>65</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E28" s="13">
         <v>1</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="G28" s="16">
-        <v>80000</v>
+        <v>25000</v>
       </c>
       <c r="H28" s="17">
         <f t="shared" si="0"/>
-        <v>80000</v>
+        <v>25000</v>
       </c>
       <c r="I28" s="13" t="s">
         <v>32</v>
       </c>
       <c r="J28" s="14" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="K28" s="15"/>
     </row>
@@ -1995,26 +1999,26 @@
         <v>65</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="E29" s="13">
         <v>1</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G29" s="16">
-        <v>70000</v>
+        <v>500000</v>
       </c>
       <c r="H29" s="17">
         <f t="shared" si="0"/>
-        <v>70000</v>
+        <v>500000</v>
       </c>
       <c r="I29" s="13" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="J29" s="14" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="K29" s="15"/>
     </row>
@@ -2023,32 +2027,32 @@
         <v>26</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C30" s="13" t="s">
         <v>65</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="E30" s="13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="G30" s="16">
-        <v>35000</v>
+        <v>160000</v>
       </c>
       <c r="H30" s="17">
         <f t="shared" si="0"/>
-        <v>175000</v>
+        <v>160000</v>
       </c>
       <c r="I30" s="13" t="s">
         <v>36</v>
       </c>
       <c r="J30" s="14" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="K30" s="15"/>
     </row>
@@ -2063,50 +2067,152 @@
         <v>65</v>
       </c>
       <c r="D31" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E31" s="13">
+        <v>1</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="G31" s="16">
+        <v>80000</v>
+      </c>
+      <c r="H31" s="17">
+        <f t="shared" si="0"/>
+        <v>80000</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="J31" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="K31" s="15"/>
+    </row>
+    <row r="32" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+      <c r="A32" s="13">
+        <v>28</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="E32" s="13">
+        <v>1</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="G32" s="16">
+        <v>70000</v>
+      </c>
+      <c r="H32" s="17">
+        <f t="shared" si="0"/>
+        <v>70000</v>
+      </c>
+      <c r="I32" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="J32" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="K32" s="15"/>
+    </row>
+    <row r="33" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+      <c r="A33" s="13">
+        <v>29</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="E33" s="13">
+        <v>5</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G33" s="16">
+        <v>35000</v>
+      </c>
+      <c r="H33" s="17">
+        <f t="shared" si="0"/>
+        <v>175000</v>
+      </c>
+      <c r="I33" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="J33" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="K33" s="15"/>
+    </row>
+    <row r="34" spans="1:11" ht="15" x14ac:dyDescent="0.3">
+      <c r="A34" s="13">
+        <v>30</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D34" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="E31" s="13">
+      <c r="E34" s="13">
         <v>2</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="F34" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="G31" s="16">
+      <c r="G34" s="16">
         <v>40000</v>
       </c>
-      <c r="H31" s="17">
-        <f t="shared" ref="H31" si="1">E31*G31</f>
+      <c r="H34" s="17">
+        <f t="shared" ref="H34" si="1">E34*G34</f>
         <v>80000</v>
       </c>
-      <c r="I31" s="13" t="s">
+      <c r="I34" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="J31" s="14" t="s">
+      <c r="J34" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="K31" s="15"/>
-    </row>
-    <row r="32" spans="1:11" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="21" t="s">
+      <c r="K34" s="15"/>
+    </row>
+    <row r="35" spans="1:11" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="19">
-        <f>SUM(H5:H31)</f>
-        <v>7990000</v>
-      </c>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="18"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="19">
+        <f>SUM(H5:H34)</f>
+        <v>11500000</v>
+      </c>
+      <c r="I35" s="18"/>
+      <c r="J35" s="18"/>
+      <c r="K35" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A35:G35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2495,15 +2601,15 @@
       <c r="K29" s="14"/>
     </row>
     <row r="30" spans="1:11" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="21" t="s">
+      <c r="A30" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="B30" s="22"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
       <c r="H30" s="19">
         <f>SUM(H5:H29)</f>
         <v>0</v>

</xml_diff>